<commit_message>
Record the POs that came before the 12 Sep delivery
The owner confirms the paid lines missing from the 12 Sep pickup lists had
already arrived:

- July's SO 1890267771 and SO 1890267773 came earlier. The backfill already
  has them as received, so they stay out of this file and the books stand.
- Infinity 3 50kg x50 (SO 1890276777), Cat Meal 20kg x15 (SO 1890276779) and
  Gravy Chunks RBL + CLS x10 each (SO 1890276783) came earlier too. They are
  now recorded as received -- stock +50, +15, +20 -- dated their SO date,
  19 Aug, since the day they arrived is not known.

Of 709 units paid for, 584 came on 12 Sep and 125 before it. Still to come:
4 -- UNO+ Grower 2, UNO+ Lactating 1, Infinity 2.1 (MP) 25x1kg 1. UNO+
Starter came 4 over. The workbook's "Not in 12 Sep delivery" sheet becomes
"Came before 12 Sep", and "Not delivered" now lists nothing.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PO Delivery Status - Sep 2026.xlsx
+++ b/PO Delivery Status - Sep 2026.xlsx
@@ -9,10 +9,11 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Came" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Not in 12 Sep delivery" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Short" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Over-delivered" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Came on older orders" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Came before 12 Sep" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Not delivered" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Short" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Over-delivered" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Came on older orders" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -46,8 +47,11 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <i val="1"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -67,16 +71,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E3F1E5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FBE0DE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EEF0F3"/>
       </patternFill>
     </fill>
   </fills>
@@ -111,7 +105,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -124,13 +118,10 @@
     <xf numFmtId="4" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="4" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -497,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -506,10 +497,11 @@
     <col width="7" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="44" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="58" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -522,7 +514,7 @@
     <row r="2" ht="44" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Paid URC sales orders (PO1–PO5.pdf) against the 12 Sep 2026 delivery (the ACI and MMFI pickup lists). "Not in 12 Sep delivery" counts every bag that did not come that day, valued at the net cost paid per bag — some of it may have come in an earlier delivery.</t>
+          <t>Paid URC sales orders (PO1–PO5.pdf). "Came 12 Sep" is the ACI and MMFI pickup lists; "Came earlier" is what the owner confirmed arrived before that delivery. "Still to come" is what is lacking, at the net cost paid.</t>
         </is>
       </c>
     </row>
@@ -559,20 +551,25 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Not in 12 Sep delivery</t>
+          <t>Came earlier</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
+          <t>Still to come</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
           <t>Amount paid</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>Value not in 12 Sep delivery</t>
-        </is>
-      </c>
       <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Value still to come</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -604,17 +601,20 @@
         <v>110</v>
       </c>
       <c r="G5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="H5" s="5" t="n">
+      <c r="I5" s="5" t="n">
         <v>183639.75</v>
       </c>
-      <c r="I5" s="5" t="n">
+      <c r="J5" s="5" t="n">
         <v>4968.24</v>
       </c>
-      <c r="J5" s="4" t="inlineStr">
-        <is>
-          <t>Partly delivered</t>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>Short — 2 Uno+ Premium Grower Pellet 50Kg/B, 1 Uno+ Premium Lactating Pellet 50kg/B</t>
         </is>
       </c>
     </row>
@@ -646,13 +646,16 @@
       <c r="G6" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="7" t="n">
+      <c r="H6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="7" t="n">
         <v>11086.5</v>
       </c>
-      <c r="I6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="6" t="inlineStr">
+      <c r="J6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="6" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -686,13 +689,16 @@
       <c r="G7" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="H7" s="7" t="n">
+      <c r="H7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="7" t="n">
         <v>40155.36</v>
       </c>
-      <c r="I7" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" s="6" t="inlineStr">
+      <c r="J7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="6" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -726,13 +732,16 @@
       <c r="G8" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="7" t="n">
+      <c r="H8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="7" t="n">
         <v>35750.4</v>
       </c>
-      <c r="I8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="6" t="inlineStr">
+      <c r="J8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="6" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -766,13 +775,16 @@
       <c r="G9" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="7" t="n">
+      <c r="H9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="7" t="n">
         <v>9416.4</v>
       </c>
-      <c r="I9" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" s="6" t="inlineStr">
+      <c r="J9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="6" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -804,97 +816,106 @@
         <v>279</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>51</v>
-      </c>
-      <c r="H10" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" s="5" t="n">
         <v>448946.25</v>
       </c>
-      <c r="I10" s="5" t="n">
-        <v>75721.92</v>
-      </c>
-      <c r="J10" s="4" t="inlineStr">
-        <is>
-          <t>Partly delivered</t>
+      <c r="J10" s="5" t="n">
+        <v>918.42</v>
+      </c>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>Short — 1 Supremo Infinity 2.1 (MP) 25x1kg</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>PO2.pdf</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>SO 1890276779</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>2026-08-19</t>
         </is>
       </c>
-      <c r="D11" s="4" t="n">
+      <c r="D11" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="E11" s="6" t="n">
         <v>45</v>
       </c>
-      <c r="F11" s="4" t="n">
+      <c r="F11" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="G11" s="4" t="n">
+      <c r="G11" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="H11" s="5" t="n">
+      <c r="H11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="7" t="n">
         <v>72700.62</v>
       </c>
-      <c r="I11" s="5" t="n">
-        <v>29236.2</v>
-      </c>
-      <c r="J11" s="4" t="inlineStr">
-        <is>
-          <t>Partly delivered</t>
+      <c r="J11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="6" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>PO2.pdf</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>SO 1890276783</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>2026-08-19</t>
         </is>
       </c>
-      <c r="D12" s="8" t="n">
+      <c r="D12" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="E12" s="8" t="n">
+      <c r="E12" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="F12" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="8" t="n">
+      <c r="F12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="H12" s="9" t="n">
+      <c r="H12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="7" t="n">
         <v>21216.16</v>
       </c>
-      <c r="I12" s="9" t="n">
-        <v>21216.2</v>
-      </c>
-      <c r="J12" s="8" t="inlineStr">
-        <is>
-          <t>None came 12 Sep</t>
+      <c r="J12" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="6" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
     </row>
@@ -926,13 +947,16 @@
       <c r="G13" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="H13" s="7" t="n">
+      <c r="H13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="7" t="n">
         <v>40155.36</v>
       </c>
-      <c r="I13" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="6" t="inlineStr">
+      <c r="J13" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="6" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -966,135 +990,148 @@
       <c r="G14" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="H14" s="7" t="n">
+      <c r="H14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="7" t="n">
         <v>62776</v>
       </c>
-      <c r="I14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="6" t="inlineStr">
+      <c r="J14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="6" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>PO5.pdf</t>
         </is>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>SO 1890267771</t>
         </is>
       </c>
-      <c r="C15" s="10" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="D15" s="10" t="n">
+      <c r="D15" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E15" s="10" t="n">
+      <c r="E15" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="F15" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" s="10" t="n">
+      <c r="F15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="H15" s="11" t="n">
+      <c r="H15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="7" t="n">
         <v>50017.5</v>
       </c>
-      <c r="I15" s="11" t="n">
-        <v>50017.6</v>
-      </c>
-      <c r="J15" s="10" t="inlineStr">
-        <is>
-          <t>None came 12 Sep — books say received earlier; confirm</t>
+      <c r="J15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="6" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>PO5.pdf</t>
         </is>
       </c>
-      <c r="B16" s="10" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>SO 1890267773</t>
         </is>
       </c>
-      <c r="C16" s="10" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="D16" s="10" t="n">
+      <c r="D16" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="E16" s="10" t="n">
+      <c r="E16" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="F16" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" s="10" t="n">
+      <c r="F16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="H16" s="11" t="n">
+      <c r="H16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="7" t="n">
         <v>8526.25</v>
       </c>
-      <c r="I16" s="11" t="n">
-        <v>8526.299999999999</v>
-      </c>
-      <c r="J16" s="10" t="inlineStr">
-        <is>
-          <t>None came 12 Sep — books say received earlier; confirm</t>
+      <c r="J16" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="6" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="inlineStr">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B17" s="13" t="n"/>
-      <c r="C17" s="13" t="n"/>
-      <c r="D17" s="12">
+      <c r="B17" s="9" t="n"/>
+      <c r="C17" s="9" t="n"/>
+      <c r="D17" s="8">
         <f>SUM(D5:D16)</f>
         <v/>
       </c>
-      <c r="E17" s="12">
+      <c r="E17" s="8">
         <f>SUM(E5:E16)</f>
         <v/>
       </c>
-      <c r="F17" s="12">
+      <c r="F17" s="8">
         <f>SUM(F5:F16)</f>
         <v/>
       </c>
-      <c r="G17" s="12">
+      <c r="G17" s="8">
         <f>SUM(G5:G16)</f>
         <v/>
       </c>
-      <c r="H17" s="14">
+      <c r="H17" s="8">
         <f>SUM(H5:H16)</f>
         <v/>
       </c>
-      <c r="I17" s="14">
+      <c r="I17" s="10">
         <f>SUM(I5:I16)</f>
         <v/>
       </c>
-      <c r="J17" s="13" t="n"/>
+      <c r="J17" s="10">
+        <f>SUM(J5:J16)</f>
+        <v/>
+      </c>
+      <c r="K17" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A2:K2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2062,29 +2099,29 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="12" t="inlineStr">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B24" s="13" t="n"/>
-      <c r="C24" s="13" t="n"/>
-      <c r="D24" s="13" t="n"/>
-      <c r="E24" s="13" t="n"/>
-      <c r="F24" s="13" t="n"/>
-      <c r="G24" s="12">
+      <c r="B24" s="9" t="n"/>
+      <c r="C24" s="9" t="n"/>
+      <c r="D24" s="9" t="n"/>
+      <c r="E24" s="9" t="n"/>
+      <c r="F24" s="9" t="n"/>
+      <c r="G24" s="8">
         <f>SUM(G5:G23)</f>
         <v/>
       </c>
-      <c r="H24" s="12">
+      <c r="H24" s="8">
         <f>SUM(H5:H23)</f>
         <v/>
       </c>
-      <c r="I24" s="12">
+      <c r="I24" s="8">
         <f>SUM(I5:I23)</f>
         <v/>
       </c>
-      <c r="J24" s="13" t="n"/>
+      <c r="J24" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2100,7 +2137,414 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:H13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="52" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Came before 12 Sep</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="44" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Not on the 12 Sep pickup lists, but confirmed by the owner to have arrived before that delivery. The day each arrived is not known; the SO date is used for it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Sales order</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>SO date</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>URC code</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Ordered</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Came</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>On the books</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>PO2.pdf</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>SO 1890276777</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>873360</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Supremo Infinity 3 (Mp) 50Kg/B</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>Recorded as received, dated 2026-08-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>PO2.pdf</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>SO 1890276779</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>878960</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>TopBreed Cat Meal 20kg</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>Recorded as received, dated 2026-08-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>PO2.pdf</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>SO 1890276783</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>879024</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>TopBreed Gravy Chunks RBL 130g (BOX)</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>Recorded as received, dated 2026-08-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>PO2.pdf</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>SO 1890276783</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>879025</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>TopBreed Gravy Chunks CLS 130g (BOX)</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>Recorded as received, dated 2026-08-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>PO5.pdf</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>SO 1890267771</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>874770</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Uno+ Supreme Lactating Pellet 50Kg/B</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>Already recorded as received (earlier backfill) — left as is</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>PO5.pdf</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>SO 1890267771</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>874720</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Uno+ Premium Breeder Pellet 50kg/B</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>Already recorded as received (earlier backfill) — left as is</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>PO5.pdf</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>SO 1890267771</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>874670</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Star Gain Starter Pellet 50Kg/B</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>Already recorded as received (earlier backfill) — left as is</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>PO5.pdf</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>SO 1890267773</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>872300</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>Supremo Infinity Ready Mix Pel Red 25kg</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>Already recorded as received (earlier backfill) — left as is</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="n"/>
+      <c r="C13" s="9" t="n"/>
+      <c r="D13" s="9" t="n"/>
+      <c r="E13" s="9" t="n"/>
+      <c r="F13" s="8">
+        <f>SUM(F5:F12)</f>
+        <v/>
+      </c>
+      <c r="G13" s="8">
+        <f>SUM(G5:G12)</f>
+        <v/>
+      </c>
+      <c r="H13" s="9" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:H2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2111,20 +2555,19 @@
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="60" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Not in 12 Sep delivery</t>
+          <t>Not delivered</t>
         </is>
       </c>
     </row>
     <row r="2" ht="44" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Paid for, but not on either 12 Sep pickup list. Missing from that delivery is not proof it never came: the "On the books" column says how each line is recorded.</t>
+          <t>Paid for and nothing of it has come, on 12 Sep or before.</t>
         </is>
       </c>
     </row>
@@ -2169,370 +2612,23 @@
           <t>Value</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>On the books</t>
-        </is>
-      </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>PO2.pdf</t>
-        </is>
-      </c>
-      <c r="B5" s="8" t="inlineStr">
-        <is>
-          <t>SO 1890276777</t>
-        </is>
-      </c>
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="D5" s="8" t="inlineStr">
-        <is>
-          <t>873360</t>
-        </is>
-      </c>
-      <c r="E5" s="8" t="inlineStr">
-        <is>
-          <t>Supremo Infinity 3 (Mp) 50Kg/B</t>
-        </is>
-      </c>
-      <c r="F5" s="8" t="n">
-        <v>50</v>
-      </c>
-      <c r="G5" s="9" t="n">
-        <v>1496.07</v>
-      </c>
-      <c r="H5" s="9" t="n">
-        <v>74803.5</v>
-      </c>
-      <c r="I5" s="8" t="inlineStr">
-        <is>
-          <t>Added as still on order (status Ordered)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>PO2.pdf</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>SO 1890276779</t>
-        </is>
-      </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>878960</t>
-        </is>
-      </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>TopBreed Cat Meal 20kg</t>
-        </is>
-      </c>
-      <c r="F6" s="8" t="n">
-        <v>15</v>
-      </c>
-      <c r="G6" s="9" t="n">
-        <v>1949.08</v>
-      </c>
-      <c r="H6" s="9" t="n">
-        <v>29236.2</v>
-      </c>
-      <c r="I6" s="8" t="inlineStr">
-        <is>
-          <t>Added as still on order (status Ordered)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>PO2.pdf</t>
-        </is>
-      </c>
-      <c r="B7" s="8" t="inlineStr">
-        <is>
-          <t>SO 1890276783</t>
-        </is>
-      </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="D7" s="8" t="inlineStr">
-        <is>
-          <t>879024</t>
-        </is>
-      </c>
-      <c r="E7" s="8" t="inlineStr">
-        <is>
-          <t>TopBreed Gravy Chunks RBL 130g (BOX)</t>
-        </is>
-      </c>
-      <c r="F7" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="G7" s="9" t="n">
-        <v>1060.81</v>
-      </c>
-      <c r="H7" s="9" t="n">
-        <v>10608.1</v>
-      </c>
-      <c r="I7" s="8" t="inlineStr">
-        <is>
-          <t>Added as still on order (status Ordered)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>PO2.pdf</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>SO 1890276783</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>879025</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>TopBreed Gravy Chunks CLS 130g (BOX)</t>
-        </is>
-      </c>
-      <c r="F8" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="G8" s="9" t="n">
-        <v>1060.81</v>
-      </c>
-      <c r="H8" s="9" t="n">
-        <v>10608.1</v>
-      </c>
-      <c r="I8" s="8" t="inlineStr">
-        <is>
-          <t>Added as still on order (status Ordered)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t>PO5.pdf</t>
-        </is>
-      </c>
-      <c r="B9" s="10" t="inlineStr">
-        <is>
-          <t>SO 1890267771</t>
-        </is>
-      </c>
-      <c r="C9" s="10" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
-      <c r="D9" s="10" t="inlineStr">
-        <is>
-          <t>874770</t>
-        </is>
-      </c>
-      <c r="E9" s="10" t="inlineStr">
-        <is>
-          <t>Uno+ Supreme Lactating Pellet 50Kg/B</t>
-        </is>
-      </c>
-      <c r="F9" s="10" t="n">
-        <v>10</v>
-      </c>
-      <c r="G9" s="11" t="n">
-        <v>1737.64</v>
-      </c>
-      <c r="H9" s="11" t="n">
-        <v>17376.4</v>
-      </c>
-      <c r="I9" s="10" t="inlineStr">
-        <is>
-          <t>Recorded as received by the earlier backfill — left as is. Confirm it came before 12 Sep.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="10" t="inlineStr">
-        <is>
-          <t>PO5.pdf</t>
-        </is>
-      </c>
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t>SO 1890267771</t>
-        </is>
-      </c>
-      <c r="C10" s="10" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
-      <c r="D10" s="10" t="inlineStr">
-        <is>
-          <t>874720</t>
-        </is>
-      </c>
-      <c r="E10" s="10" t="inlineStr">
-        <is>
-          <t>Uno+ Premium Breeder Pellet 50kg/B</t>
-        </is>
-      </c>
-      <c r="F10" s="10" t="n">
-        <v>10</v>
-      </c>
-      <c r="G10" s="11" t="n">
-        <v>1588.07</v>
-      </c>
-      <c r="H10" s="11" t="n">
-        <v>15880.7</v>
-      </c>
-      <c r="I10" s="10" t="inlineStr">
-        <is>
-          <t>Recorded as received by the earlier backfill — left as is. Confirm it came before 12 Sep.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>PO5.pdf</t>
-        </is>
-      </c>
-      <c r="B11" s="10" t="inlineStr">
-        <is>
-          <t>SO 1890267771</t>
-        </is>
-      </c>
-      <c r="C11" s="10" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
-      <c r="D11" s="10" t="inlineStr">
-        <is>
-          <t>874670</t>
-        </is>
-      </c>
-      <c r="E11" s="10" t="inlineStr">
-        <is>
-          <t>Star Gain Starter Pellet 50Kg/B</t>
-        </is>
-      </c>
-      <c r="F11" s="10" t="n">
-        <v>10</v>
-      </c>
-      <c r="G11" s="11" t="n">
-        <v>1676.05</v>
-      </c>
-      <c r="H11" s="11" t="n">
-        <v>16760.5</v>
-      </c>
-      <c r="I11" s="10" t="inlineStr">
-        <is>
-          <t>Recorded as received by the earlier backfill — left as is. Confirm it came before 12 Sep.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="10" t="inlineStr">
-        <is>
-          <t>PO5.pdf</t>
-        </is>
-      </c>
-      <c r="B12" s="10" t="inlineStr">
-        <is>
-          <t>SO 1890267773</t>
-        </is>
-      </c>
-      <c r="C12" s="10" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
-      <c r="D12" s="10" t="inlineStr">
-        <is>
-          <t>872300</t>
-        </is>
-      </c>
-      <c r="E12" s="10" t="inlineStr">
-        <is>
-          <t>Supremo Infinity Ready Mix Pel Red 25kg</t>
-        </is>
-      </c>
-      <c r="F12" s="10" t="n">
-        <v>10</v>
-      </c>
-      <c r="G12" s="11" t="n">
-        <v>852.63</v>
-      </c>
-      <c r="H12" s="11" t="n">
-        <v>8526.299999999999</v>
-      </c>
-      <c r="I12" s="10" t="inlineStr">
-        <is>
-          <t>Recorded as received by the earlier backfill — left as is. Confirm it came before 12 Sep.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="12" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B13" s="13" t="n"/>
-      <c r="C13" s="13" t="n"/>
-      <c r="D13" s="13" t="n"/>
-      <c r="E13" s="13" t="n"/>
-      <c r="F13" s="12">
-        <f>SUM(F5:F12)</f>
-        <v/>
-      </c>
-      <c r="G13" s="13" t="n"/>
-      <c r="H13" s="14">
-        <f>SUM(H5:H12)</f>
-        <v/>
-      </c>
-      <c r="I13" s="13" t="n"/>
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A2:H2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2725,28 +2821,28 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B8" s="13" t="n"/>
-      <c r="C8" s="13" t="n"/>
-      <c r="D8" s="13" t="n"/>
-      <c r="E8" s="12">
+      <c r="B8" s="9" t="n"/>
+      <c r="C8" s="9" t="n"/>
+      <c r="D8" s="9" t="n"/>
+      <c r="E8" s="8">
         <f>SUM(E5:E7)</f>
         <v/>
       </c>
-      <c r="F8" s="12">
+      <c r="F8" s="8">
         <f>SUM(F5:F7)</f>
         <v/>
       </c>
-      <c r="G8" s="12">
+      <c r="G8" s="8">
         <f>SUM(G5:G7)</f>
         <v/>
       </c>
-      <c r="H8" s="13" t="n"/>
-      <c r="I8" s="14">
+      <c r="H8" s="9" t="n"/>
+      <c r="I8" s="10">
         <f>SUM(I5:I7)</f>
         <v/>
       </c>
@@ -2759,7 +2855,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2849,22 +2945,22 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B6" s="13" t="n"/>
-      <c r="C6" s="13" t="n"/>
-      <c r="D6" s="12">
+      <c r="B6" s="9" t="n"/>
+      <c r="C6" s="9" t="n"/>
+      <c r="D6" s="8">
         <f>SUM(D5:D5)</f>
         <v/>
       </c>
-      <c r="E6" s="12">
+      <c r="E6" s="8">
         <f>SUM(E5:E5)</f>
         <v/>
       </c>
-      <c r="F6" s="12">
+      <c r="F6" s="8">
         <f>SUM(F5:F5)</f>
         <v/>
       </c>
@@ -2877,7 +2973,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2947,227 +3043,227 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>ACI</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>07-Sep</t>
         </is>
       </c>
-      <c r="C5" s="15" t="inlineStr">
+      <c r="C5" s="12" t="inlineStr">
         <is>
           <t>SO 1890279846</t>
         </is>
       </c>
-      <c r="D5" s="15" t="inlineStr">
+      <c r="D5" s="12" t="inlineStr">
         <is>
           <t>SO 1890274632</t>
         </is>
       </c>
-      <c r="E5" s="15" t="inlineStr">
+      <c r="E5" s="12" t="inlineStr">
         <is>
           <t>871130</t>
         </is>
       </c>
-      <c r="F5" s="15" t="inlineStr">
+      <c r="F5" s="12" t="inlineStr">
         <is>
           <t>Supremo Infinity 2 (CGC) 25x1kg</t>
         </is>
       </c>
-      <c r="G5" s="15" t="n">
+      <c r="G5" s="12" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>ACI</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>07-Sep</t>
         </is>
       </c>
-      <c r="C6" s="15" t="inlineStr">
+      <c r="C6" s="12" t="inlineStr">
         <is>
           <t>SO 1890279846</t>
         </is>
       </c>
-      <c r="D6" s="15" t="inlineStr">
+      <c r="D6" s="12" t="inlineStr">
         <is>
           <t>SO 1890274632</t>
         </is>
       </c>
-      <c r="E6" s="15" t="inlineStr">
+      <c r="E6" s="12" t="inlineStr">
         <is>
           <t>871140</t>
         </is>
       </c>
-      <c r="F6" s="15" t="inlineStr">
+      <c r="F6" s="12" t="inlineStr">
         <is>
           <t>Supremo Infinity 2.1 (MP) 25x1kg</t>
         </is>
       </c>
-      <c r="G6" s="15" t="n">
+      <c r="G6" s="12" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>ACI</t>
         </is>
       </c>
-      <c r="B7" s="15" t="inlineStr">
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>07-Sep</t>
         </is>
       </c>
-      <c r="C7" s="15" t="inlineStr">
+      <c r="C7" s="12" t="inlineStr">
         <is>
           <t>SO 1890279846</t>
         </is>
       </c>
-      <c r="D7" s="15" t="inlineStr">
+      <c r="D7" s="12" t="inlineStr">
         <is>
           <t>SO 1890274632</t>
         </is>
       </c>
-      <c r="E7" s="15" t="inlineStr">
+      <c r="E7" s="12" t="inlineStr">
         <is>
           <t>871150</t>
         </is>
       </c>
-      <c r="F7" s="15" t="inlineStr">
+      <c r="F7" s="12" t="inlineStr">
         <is>
           <t>Supremo Infinity 4 (BP) 25x1kg</t>
         </is>
       </c>
-      <c r="G7" s="15" t="n">
+      <c r="G7" s="12" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>ACI</t>
         </is>
       </c>
-      <c r="B8" s="15" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>07-Sep</t>
         </is>
       </c>
-      <c r="C8" s="15" t="inlineStr">
+      <c r="C8" s="12" t="inlineStr">
         <is>
           <t>SO 1890279846</t>
         </is>
       </c>
-      <c r="D8" s="15" t="inlineStr">
+      <c r="D8" s="12" t="inlineStr">
         <is>
           <t>SO 1890274632</t>
         </is>
       </c>
-      <c r="E8" s="15" t="inlineStr">
+      <c r="E8" s="12" t="inlineStr">
         <is>
           <t>872430</t>
         </is>
       </c>
-      <c r="F8" s="15" t="inlineStr">
+      <c r="F8" s="12" t="inlineStr">
         <is>
           <t>Supremo Infinity Fortifier 32 HPP 25x1kg</t>
         </is>
       </c>
-      <c r="G8" s="15" t="n">
+      <c r="G8" s="12" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>ACI</t>
         </is>
       </c>
-      <c r="B9" s="15" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>07-Aug</t>
         </is>
       </c>
-      <c r="C9" s="15" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
         <is>
           <t>SO 1890274638</t>
         </is>
       </c>
-      <c r="D9" s="15" t="inlineStr">
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>(same)</t>
         </is>
       </c>
-      <c r="E9" s="15" t="inlineStr">
+      <c r="E9" s="12" t="inlineStr">
         <is>
           <t>878590</t>
         </is>
       </c>
-      <c r="F9" s="15" t="inlineStr">
+      <c r="F9" s="12" t="inlineStr">
         <is>
           <t>Topbreed 5Kg Adult Dog Meal</t>
         </is>
       </c>
-      <c r="G9" s="15" t="n">
+      <c r="G9" s="12" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="15" t="inlineStr">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>ACI</t>
         </is>
       </c>
-      <c r="B10" s="15" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>24-Jul</t>
         </is>
       </c>
-      <c r="C10" s="15" t="inlineStr">
+      <c r="C10" s="12" t="inlineStr">
         <is>
           <t>SO 1890271973</t>
         </is>
       </c>
-      <c r="D10" s="15" t="inlineStr">
+      <c r="D10" s="12" t="inlineStr">
         <is>
           <t>(same)</t>
         </is>
       </c>
-      <c r="E10" s="15" t="inlineStr">
+      <c r="E10" s="12" t="inlineStr">
         <is>
           <t>878590</t>
         </is>
       </c>
-      <c r="F10" s="15" t="inlineStr">
+      <c r="F10" s="12" t="inlineStr">
         <is>
           <t>Topbreed 5Kg Adult Dog Meal</t>
         </is>
       </c>
-      <c r="G10" s="15" t="n">
+      <c r="G10" s="12" t="n">
         <v>35</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B11" s="13" t="n"/>
-      <c r="C11" s="13" t="n"/>
-      <c r="D11" s="13" t="n"/>
-      <c r="E11" s="13" t="n"/>
-      <c r="F11" s="13" t="n"/>
-      <c r="G11" s="12">
+      <c r="B11" s="9" t="n"/>
+      <c r="C11" s="9" t="n"/>
+      <c r="D11" s="9" t="n"/>
+      <c r="E11" s="9" t="n"/>
+      <c r="F11" s="9" t="n"/>
+      <c r="G11" s="8">
         <f>SUM(G5:G10)</f>
         <v/>
       </c>

</xml_diff>